<commit_message>
Corregir reacción de apoyos inferiores en memoria combinada y resultados
La lectura directa de los nodos del apoyo inferior omite la presión
aplicada sobre el propio parche (~1.5 kN por g). La reacción se toma
ahora por equilibrio horizontal con las orejas: B0 117 kN a 3g,
P3 +29 %, P4 +44 %. El Excel incluye ambas lecturas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TixyxqUNmuV7iGi3jJYj2g
</commit_message>
<xml_diff>
--- a/Resultados_FEA_reconstruido.xlsx
+++ b/Resultados_FEA_reconstruido.xlsx
@@ -1610,7 +1610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1731,84 +1731,112 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Apoyos inferiores, suma eje X, 3g (kN)</t>
+          <t>Apoyos inferiores, suma eje X, 3g, por equilibrio con las orejas (kN)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>112.50975</v>
+        <v>116.97825</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>136.54014</v>
+        <v>140.97063</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>136.13175</v>
+        <v>140.8989</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>137.15733</v>
+        <v>141.62568</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>136.81434</v>
+        <v>141.62589</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>145.65645</v>
+        <v>150.49137</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>164.14605</v>
+        <v>168.61491</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mínima compresión apoyo inferior, todos los casos (kN)</t>
+          <t>Apoyos inferiores, suma eje X, 3g, lectura directa de nodos (omite la presión sobre el parche) (kN)</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>7.203225000000003</v>
+        <v>112.50975</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10.309175</v>
+        <v>136.54014</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>9.068894999999998</v>
+        <v>136.13175</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>10.43818</v>
+        <v>137.15733</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>7.440019999999999</v>
+        <v>136.81434</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>9.102105</v>
+        <v>145.65645</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>11.729825</v>
+        <v>164.14605</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Mínima compresión apoyo inferior, todos los casos (kN)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7.203225000000003</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>10.309175</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>9.068894999999998</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>10.43818</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>7.440019999999999</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>9.102105</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>11.729825</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Suma de reacciones verticales a 1g (kN)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B9" s="3" t="n">
         <v>67.46627767999999</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C9" s="3" t="n">
         <v>80.63253816000001</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D9" s="3" t="n">
         <v>80.41604963999998</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E9" s="3" t="n">
         <v>82.17015767999999</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F9" s="3" t="n">
         <v>81.95362935000001</v>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G9" s="3" t="n">
         <v>81.90011935000001</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H9" s="3" t="n">
         <v>83.35760767999999</v>
       </c>
     </row>

</xml_diff>